<commit_message>
increate limit search from 30 to 100
</commit_message>
<xml_diff>
--- a/output/small.xlsx
+++ b/output/small.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Documents/Projects/AI/find-price/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB51A8F-79BF-224E-8378-B46F3BE6B8E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B02CE58-8E53-A54F-B28D-9F170BBD92E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4700" yWindow="760" windowWidth="25640" windowHeight="14440" activeTab="1" xr2:uid="{F2CA0B74-71ED-EA4D-A14D-BFD29DF0BB1C}"/>
+    <workbookView xWindow="4600" yWindow="760" windowWidth="25640" windowHeight="14440" activeTab="1" xr2:uid="{F2CA0B74-71ED-EA4D-A14D-BFD29DF0BB1C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>